<commit_message>
feat: implement record metadata extracting functionality
</commit_message>
<xml_diff>
--- a/Reports/Test/expenses.xlsx
+++ b/Reports/Test/expenses.xlsx
@@ -367,7 +367,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2">
-        <v>46175.604166666664</v>
+        <v>46174.375</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>7</v>
@@ -381,7 +381,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2">
-        <v>46178.427083333336</v>
+        <v>46174.375</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>9</v>
@@ -398,7 +398,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2">
-        <v>46183.458333333336</v>
+        <v>46174.375</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>7</v>
@@ -412,7 +412,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2">
-        <v>46187.697916666664</v>
+        <v>46174.375</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>13</v>
@@ -429,7 +429,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2">
-        <v>46193.354166666664</v>
+        <v>46174.375</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>16</v>
@@ -443,7 +443,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2">
-        <v>46201.555555555555</v>
+        <v>46174.375</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>9</v>

</xml_diff>